<commit_message>
:herb::herb: div. script run w F60 data
</commit_message>
<xml_diff>
--- a/data/derived_data/4_Diversities/ps_16S_rare_expe_D1_otu_table.xlsx
+++ b/data/derived_data/4_Diversities/ps_16S_rare_expe_D1_otu_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -38,12 +38,21 @@
     <t xml:space="preserve">MS_025</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_027</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_028</t>
   </si>
   <si>
     <t xml:space="preserve">MS_030</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_032</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_035</t>
   </si>
   <si>
@@ -56,6 +65,9 @@
     <t xml:space="preserve">MS_038</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_039</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_040</t>
   </si>
   <si>
@@ -77,6 +89,12 @@
     <t xml:space="preserve">MS_060</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_064</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_065</t>
   </si>
   <si>
@@ -98,12 +116,39 @@
     <t xml:space="preserve">MS_072</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_087</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_090</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_091</t>
   </si>
   <si>
     <t xml:space="preserve">MS_092</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_093</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_097</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_100</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_101</t>
   </si>
   <si>
@@ -155,6 +200,9 @@
     <t xml:space="preserve">MS_137</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_138</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_141</t>
   </si>
   <si>
@@ -170,6 +218,9 @@
     <t xml:space="preserve">MS_146</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_153</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_155</t>
   </si>
   <si>
@@ -200,6 +251,9 @@
     <t xml:space="preserve">MS_166</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_168</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_169</t>
   </si>
   <si>
@@ -212,6 +266,9 @@
     <t xml:space="preserve">MS_173</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_265</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_266</t>
   </si>
   <si>
@@ -221,6 +278,9 @@
     <t xml:space="preserve">MS_268</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_269</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_271</t>
   </si>
   <si>
@@ -230,22 +290,34 @@
     <t xml:space="preserve">MS_273</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_11</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_113</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_14</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_16</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_17</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_20</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_23</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_31</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_34</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_5</t>
@@ -809,16 +881,76 @@
       <c r="BT1" t="s">
         <v>71</v>
       </c>
+      <c r="BU1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" t="s">
+        <v>87</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>89</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>90</v>
+      </c>
+      <c r="CN1" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -827,28 +959,28 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>822</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>2809</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>619</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>2810</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -914,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0</v>
+        <v>861</v>
       </c>
       <c r="AK2" t="n">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="AL2" t="n">
         <v>0</v>
@@ -932,13 +1064,13 @@
         <v>0</v>
       </c>
       <c r="AO2" t="n">
-        <v>0</v>
+        <v>1346</v>
       </c>
       <c r="AP2" t="n">
-        <v>0</v>
+        <v>723</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0</v>
+        <v>2593</v>
       </c>
       <c r="AR2" t="n">
         <v>0</v>
@@ -1025,24 +1157,84 @@
         <v>0</v>
       </c>
       <c r="BT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>1590</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>1190</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>30</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>83</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>2753</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="B3" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>231</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -1084,7 +1276,7 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
@@ -1093,16 +1285,16 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="W3" t="n">
-        <v>7</v>
+        <v>227</v>
       </c>
       <c r="X3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
         <v>0</v>
@@ -1117,16 +1309,16 @@
         <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="AF3" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="AH3" t="n">
         <v>0</v>
@@ -1138,10 +1330,10 @@
         <v>0</v>
       </c>
       <c r="AK3" t="n">
-        <v>0</v>
+        <v>1412</v>
       </c>
       <c r="AL3" t="n">
-        <v>0</v>
+        <v>2832</v>
       </c>
       <c r="AM3" t="n">
         <v>0</v>
@@ -1150,7 +1342,7 @@
         <v>0</v>
       </c>
       <c r="AO3" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="AP3" t="n">
         <v>0</v>
@@ -1159,16 +1351,16 @@
         <v>0</v>
       </c>
       <c r="AR3" t="n">
-        <v>0</v>
+        <v>1925</v>
       </c>
       <c r="AS3" t="n">
-        <v>0</v>
+        <v>1639</v>
       </c>
       <c r="AT3" t="n">
-        <v>0</v>
+        <v>567</v>
       </c>
       <c r="AU3" t="n">
-        <v>0</v>
+        <v>824</v>
       </c>
       <c r="AV3" t="n">
         <v>0</v>
@@ -1180,13 +1372,13 @@
         <v>0</v>
       </c>
       <c r="AY3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="AZ3" t="n">
         <v>0</v>
       </c>
       <c r="BA3" t="n">
-        <v>0</v>
+        <v>784</v>
       </c>
       <c r="BB3" t="n">
         <v>0</v>
@@ -1216,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="BK3" t="n">
-        <v>0</v>
+        <v>2730</v>
       </c>
       <c r="BL3" t="n">
         <v>0</v>
@@ -1228,13 +1420,13 @@
         <v>0</v>
       </c>
       <c r="BO3" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="BP3" t="n">
         <v>0</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0</v>
+        <v>2126</v>
       </c>
       <c r="BR3" t="n">
         <v>0</v>
@@ -1243,18 +1435,78 @@
         <v>0</v>
       </c>
       <c r="BT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB3" t="n">
+        <v>477</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>15</v>
+      </c>
+      <c r="CM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1263,7 +1515,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1275,7 +1527,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1299,37 +1551,37 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>153</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
@@ -1338,16 +1590,16 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="AI4" t="n">
         <v>0</v>
@@ -1359,10 +1611,10 @@
         <v>0</v>
       </c>
       <c r="AL4" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1389,13 +1641,13 @@
         <v>0</v>
       </c>
       <c r="AV4" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="AW4" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="AX4" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="AY4" t="n">
         <v>0</v>
@@ -1413,7 +1665,7 @@
         <v>0</v>
       </c>
       <c r="BD4" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="BE4" t="n">
         <v>0</v>
@@ -1431,16 +1683,16 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="BK4" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="BL4" t="n">
         <v>0</v>
       </c>
       <c r="BM4" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="BN4" t="n">
         <v>0</v>
@@ -1452,27 +1704,87 @@
         <v>0</v>
       </c>
       <c r="BQ4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="BR4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="BS4" t="n">
         <v>0</v>
       </c>
       <c r="BT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1499,28 +1811,28 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>363</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>393</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>401</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
@@ -1541,10 +1853,10 @@
         <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="AA5" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="AB5" t="n">
         <v>0</v>
@@ -1553,7 +1865,7 @@
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1589,7 +1901,7 @@
         <v>0</v>
       </c>
       <c r="AP5" t="n">
-        <v>0</v>
+        <v>2250</v>
       </c>
       <c r="AQ5" t="n">
         <v>0</v>
@@ -1601,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="AT5" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="AU5" t="n">
         <v>0</v>
@@ -1679,24 +1991,84 @@
         <v>0</v>
       </c>
       <c r="BT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>94</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>235</v>
       </c>
       <c r="E6" t="n">
-        <v>21</v>
+        <v>261</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -1723,40 +2095,40 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
         <v>1</v>
       </c>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
       <c r="X6" t="n">
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
@@ -1765,16 +2137,16 @@
         <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AC6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AD6" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AE6" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AF6" t="n">
         <v>0</v>
@@ -1792,10 +2164,10 @@
         <v>0</v>
       </c>
       <c r="AK6" t="n">
-        <v>0</v>
+        <v>1260</v>
       </c>
       <c r="AL6" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="AM6" t="n">
         <v>0</v>
@@ -1897,12 +2269,72 @@
         <v>0</v>
       </c>
       <c r="BT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -1911,10 +2343,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1953,7 +2385,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
@@ -2001,7 +2433,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="AI7" t="n">
         <v>0</v>
@@ -2022,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="AO7" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="AP7" t="n">
         <v>0</v>
@@ -2067,10 +2499,10 @@
         <v>0</v>
       </c>
       <c r="BD7" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="BE7" t="n">
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="BF7" t="n">
         <v>0</v>
@@ -2116,229 +2548,349 @@
       </c>
       <c r="BT7" t="n">
         <v>0</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>961</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>26</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>155</v>
+      </c>
+      <c r="W8" t="n">
+        <v>147</v>
+      </c>
+      <c r="X8" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>27</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>54</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>115</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>123</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>57</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>11</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>14</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>49</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>58</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>124</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>106</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>83</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>77</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>72</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>72</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>63</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>50</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>132</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA8" t="n">
         <v>78</v>
       </c>
-      <c r="B8" t="n">
-        <v>2942</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2876</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2756</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2559</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2959</v>
-      </c>
-      <c r="G8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="H8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="I8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J8" t="n">
-        <v>2606</v>
-      </c>
-      <c r="K8" t="n">
-        <v>2808</v>
-      </c>
-      <c r="L8" t="n">
-        <v>2572</v>
-      </c>
-      <c r="M8" t="n">
-        <v>519</v>
-      </c>
-      <c r="N8" t="n">
-        <v>2727</v>
-      </c>
-      <c r="O8" t="n">
-        <v>2564</v>
-      </c>
-      <c r="P8" t="n">
-        <v>2602</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>2714</v>
-      </c>
-      <c r="R8" t="n">
-        <v>1830</v>
-      </c>
-      <c r="S8" t="n">
-        <v>1859</v>
-      </c>
-      <c r="T8" t="n">
-        <v>1831</v>
-      </c>
-      <c r="U8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="V8" t="n">
-        <v>1745</v>
-      </c>
-      <c r="W8" t="n">
-        <v>1884</v>
-      </c>
-      <c r="X8" t="n">
-        <v>1312</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>1763</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>1016</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>979</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>444</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>776</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>706</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>320</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>789</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>39</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>235</v>
-      </c>
-      <c r="AW8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO8" t="n">
-        <v>1230</v>
-      </c>
-      <c r="BP8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="BQ8" t="n">
-        <v>2238</v>
-      </c>
-      <c r="BR8" t="n">
-        <v>2562</v>
-      </c>
-      <c r="BS8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="BT8" t="n">
-        <v>2559</v>
+      <c r="CB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>111</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>92</v>
+      </c>
+      <c r="CF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>35</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>2</v>
+      </c>
+      <c r="CM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -2350,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>151</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -2536,10 +3088,10 @@
         <v>0</v>
       </c>
       <c r="BO9" t="n">
-        <v>0</v>
+        <v>196</v>
       </c>
       <c r="BP9" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="BQ9" t="n">
         <v>0</v>
@@ -2551,18 +3103,78 @@
         <v>0</v>
       </c>
       <c r="BT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -2583,7 +3195,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -2595,163 +3207,163 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>397</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>286</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>1161</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>1194</v>
+        <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>1245</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>1108</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="n">
         <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>1581</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>1605</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>2394</v>
+        <v>0</v>
       </c>
       <c r="AC10" t="n">
-        <v>3000</v>
+        <v>1</v>
       </c>
       <c r="AD10" t="n">
-        <v>2224</v>
+        <v>0</v>
       </c>
       <c r="AE10" t="n">
-        <v>669</v>
+        <v>0</v>
       </c>
       <c r="AF10" t="n">
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>2404</v>
+        <v>0</v>
       </c>
       <c r="AI10" t="n">
-        <v>2294</v>
+        <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>2680</v>
+        <v>0</v>
       </c>
       <c r="AK10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AL10" t="n">
-        <v>1821</v>
+        <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>676</v>
+        <v>0</v>
       </c>
       <c r="AN10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AO10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>2211</v>
+        <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>2961</v>
+        <v>0</v>
       </c>
       <c r="AT10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AU10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AV10" t="n">
-        <v>2530</v>
+        <v>0</v>
       </c>
       <c r="AW10" t="n">
-        <v>676</v>
+        <v>0</v>
       </c>
       <c r="AX10" t="n">
-        <v>483</v>
+        <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AZ10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BA10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BB10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BC10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BD10" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="BE10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BG10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BH10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BI10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BJ10" t="n">
-        <v>798</v>
+        <v>0</v>
       </c>
       <c r="BK10" t="n">
-        <v>1894</v>
+        <v>0</v>
       </c>
       <c r="BL10" t="n">
-        <v>2870</v>
+        <v>0</v>
       </c>
       <c r="BM10" t="n">
-        <v>2640</v>
+        <v>0</v>
       </c>
       <c r="BN10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BO10" t="n">
         <v>0</v>
@@ -2760,33 +3372,93 @@
         <v>0</v>
       </c>
       <c r="BQ10" t="n">
-        <v>517</v>
+        <v>0</v>
       </c>
       <c r="BR10" t="n">
-        <v>401</v>
+        <v>0</v>
       </c>
       <c r="BS10" t="n">
         <v>0</v>
       </c>
       <c r="BT10" t="n">
-        <v>404</v>
+        <v>0</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -2801,34 +3473,34 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>192</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>428</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>2481</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>436</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R11" t="n">
-        <v>963</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>867</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
@@ -2837,25 +3509,25 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>1630</v>
+        <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>1161</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="AB11" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
@@ -2864,16 +3536,16 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>494</v>
+        <v>0</v>
       </c>
       <c r="AF11" t="n">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="AG11" t="n">
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>501</v>
+        <v>0</v>
       </c>
       <c r="AI11" t="n">
         <v>0</v>
@@ -2888,7 +3560,7 @@
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>197</v>
+        <v>0</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2939,7 +3611,7 @@
         <v>0</v>
       </c>
       <c r="BD11" t="n">
-        <v>1998</v>
+        <v>0</v>
       </c>
       <c r="BE11" t="n">
         <v>0</v>
@@ -2972,13 +3644,13 @@
         <v>0</v>
       </c>
       <c r="BO11" t="n">
-        <v>1770</v>
+        <v>0</v>
       </c>
       <c r="BP11" t="n">
         <v>0</v>
       </c>
       <c r="BQ11" t="n">
-        <v>195</v>
+        <v>0</v>
       </c>
       <c r="BR11" t="n">
         <v>0</v>
@@ -2987,33 +3659,93 @@
         <v>0</v>
       </c>
       <c r="BT11" t="n">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>2950</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>2891</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>2765</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>2560</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2962</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2178</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>2938</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -3022,49 +3754,49 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2929</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>2021</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>2802</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>2238</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>501</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>2708</v>
       </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>2744</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>2197</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>2591</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>2717</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>1674</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>1711</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>1843</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>1851</v>
       </c>
       <c r="Z12" t="n">
         <v>0</v>
@@ -3073,31 +3805,31 @@
         <v>0</v>
       </c>
       <c r="AB12" t="n">
-        <v>0</v>
+        <v>1763</v>
       </c>
       <c r="AC12" t="n">
-        <v>0</v>
+        <v>1910</v>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>1301</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>1772</v>
       </c>
       <c r="AF12" t="n">
-        <v>0</v>
+        <v>1028</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>983</v>
       </c>
       <c r="AH12" t="n">
-        <v>0</v>
+        <v>457</v>
       </c>
       <c r="AI12" t="n">
         <v>0</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0</v>
+        <v>2139</v>
       </c>
       <c r="AK12" t="n">
         <v>0</v>
@@ -3109,22 +3841,22 @@
         <v>0</v>
       </c>
       <c r="AN12" t="n">
-        <v>0</v>
+        <v>763</v>
       </c>
       <c r="AO12" t="n">
-        <v>0</v>
+        <v>1015</v>
       </c>
       <c r="AP12" t="n">
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="AR12" t="n">
-        <v>0</v>
+        <v>746</v>
       </c>
       <c r="AS12" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="AT12" t="n">
         <v>0</v>
@@ -3139,10 +3871,10 @@
         <v>0</v>
       </c>
       <c r="AX12" t="n">
-        <v>0</v>
+        <v>725</v>
       </c>
       <c r="AY12" t="n">
-        <v>0</v>
+        <v>344</v>
       </c>
       <c r="AZ12" t="n">
         <v>0</v>
@@ -3160,7 +3892,7 @@
         <v>0</v>
       </c>
       <c r="BE12" t="n">
-        <v>0</v>
+        <v>678</v>
       </c>
       <c r="BF12" t="n">
         <v>0</v>
@@ -3169,7 +3901,7 @@
         <v>0</v>
       </c>
       <c r="BH12" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="BI12" t="n">
         <v>0</v>
@@ -3181,7 +3913,7 @@
         <v>0</v>
       </c>
       <c r="BL12" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="BM12" t="n">
         <v>0</v>
@@ -3206,11 +3938,71 @@
       </c>
       <c r="BT12" t="n">
         <v>0</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH12" t="n">
+        <v>703</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>2970</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>2184</v>
+      </c>
+      <c r="CK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL12" t="n">
+        <v>2569</v>
+      </c>
+      <c r="CM12" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CN12" t="n">
+        <v>2473</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -3222,7 +4014,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -3285,144 +4077,1316 @@
         <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="AA13" t="n">
-        <v>241</v>
+        <v>0</v>
       </c>
       <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>21</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>27</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>40</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>19</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>183</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>287</v>
+      </c>
+      <c r="R14" t="n">
+        <v>122</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>409</v>
+      </c>
+      <c r="U14" t="n">
+        <v>282</v>
+      </c>
+      <c r="V14" t="n">
+        <v>49</v>
+      </c>
+      <c r="W14" t="n">
+        <v>81</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1151</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>1142</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>1221</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>1082</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>1532</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>1529</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>2157</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>2237</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>306</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>71</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>522</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>2334</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>2275</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>2615</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>1345</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>647</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>2976</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>1840</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>2954</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>270</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>2573</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>626</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>486</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>2625</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>2956</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>651</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>940</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BY14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CA14" t="n">
+        <v>780</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>2523</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>1948</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>2870</v>
+      </c>
+      <c r="CE14" t="n">
+        <v>2636</v>
+      </c>
+      <c r="CF14" t="n">
+        <v>2039</v>
+      </c>
+      <c r="CG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>499</v>
+      </c>
+      <c r="CK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL14" t="n">
+        <v>385</v>
+      </c>
+      <c r="CM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN14" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>191</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>130</v>
+      </c>
+      <c r="M15" t="n">
+        <v>190</v>
+      </c>
+      <c r="N15" t="n">
+        <v>156</v>
+      </c>
+      <c r="O15" t="n">
+        <v>399</v>
+      </c>
+      <c r="P15" t="n">
+        <v>2106</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>402</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="n">
+        <v>939</v>
+      </c>
+      <c r="W15" t="n">
+        <v>833</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="n">
         <v>1</v>
       </c>
-      <c r="AC13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>1782</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>2591</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>1078</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>2052</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>163</v>
-      </c>
-      <c r="AW13" t="n">
-        <v>2255</v>
-      </c>
-      <c r="AX13" t="n">
-        <v>2438</v>
-      </c>
-      <c r="AY13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>2126</v>
-      </c>
-      <c r="BK13" t="n">
-        <v>990</v>
-      </c>
-      <c r="BL13" t="n">
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>1562</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>1068</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>49</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>54</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>92</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>65</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>122</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>361</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>204</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>960</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>410</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>184</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>560</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>205</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>106</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>1928</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG15" t="n">
+        <v>1410</v>
+      </c>
+      <c r="CH15" t="n">
+        <v>1013</v>
+      </c>
+      <c r="CI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ15" t="n">
+        <v>199</v>
+      </c>
+      <c r="CK15" t="n">
+        <v>247</v>
+      </c>
+      <c r="CL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN15" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>211</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>240</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>1417</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>1868</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>788</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>2071</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>145</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>2302</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>2451</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>67</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA17" t="n">
+        <v>2142</v>
+      </c>
+      <c r="CB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC17" t="n">
+        <v>941</v>
+      </c>
+      <c r="CD17" t="n">
         <v>130</v>
       </c>
-      <c r="BM13" t="n">
-        <v>289</v>
-      </c>
-      <c r="BN13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR13" t="n">
+      <c r="CE17" t="n">
+        <v>272</v>
+      </c>
+      <c r="CF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL17" t="n">
         <v>29</v>
       </c>
-      <c r="BS13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT13" t="n">
+      <c r="CM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>